<commit_message>
updated veg 2023 dataframes, exported as excel to folder = summary output, ready to read into slash_veg_complete.Rmd
</commit_message>
<xml_diff>
--- a/where to start coding - notes from the last session.xlsx
+++ b/where to start coding - notes from the last session.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F2468D0-CE2E-41A6-A986-6A28AF746AED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06FAA6F-033B-4501-98A2-53386AAA4F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Date of Coding</t>
   </si>
@@ -59,13 +59,22 @@
     <t>line 1000 - how to input the basal area data for 2023 or 2024 to give a complete picture of the site variables. Run through to make data complete. Schedule with stat consulting.</t>
   </si>
   <si>
-    <t>july 28 2025</t>
-  </si>
-  <si>
     <t xml:space="preserve">the site data were all combined into a full data frame 2019 - 2024. </t>
   </si>
   <si>
     <t>line 1452 df=regen2023 and df=regen2024 need to be reconfigured to mesh with df=2019-2022 and then made complete.  calculations of clump dta are only possible for the 2023 and 2024 data. Line 400 df=regen2023 needs to read the raw data used in file="test_2023_regen_plot_input.Rmd" to make calculations of trees per acre for single and clumps, and the calculate clumps per acre and average stems per ramet. There are two datafiles to read at line 128 and 194.  The equations of these calculations and the code are done for df=regen2024 line 469 and can likely be copied.</t>
+  </si>
+  <si>
+    <t>july 18 2025</t>
+  </si>
+  <si>
+    <t>july 19 2025</t>
+  </si>
+  <si>
+    <t>revise and output the 2023 veg data in raw format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The 2023 veg data was exported, raw without manipulation, into folder "summary output" as df = "veg2023_raw(19july2025)" from file="test_2023_regen_plot_input.Rmd".  Read that data into "slash_veg_complete.Rmd" at line 416 and calculate the stems per acre and "clumps_per acre" and "ramets_clump". Check the plot radius coefficients on line 407 The code for the clump and ramet calculations are likely available on line ~469 for df=veg2024 and have been confirmed.  </t>
   </si>
 </sst>
 </file>
@@ -75,8 +84,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -104,11 +121,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -118,6 +132,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,30 +476,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10441F4B-E333-43AC-9DFC-8056F26DEB96}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="62.7109375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="78" style="4" customWidth="1"/>
+    <col min="2" max="2" width="62.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="78" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" s="4" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="3" spans="1:3" s="3" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
         <v>45852</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -483,25 +507,37 @@
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="148.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>9</v>
+    </row>
+    <row r="6" spans="1:3" ht="125.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
reworking the data, especially regen2023 and regen2024. fine tuning teh blending.
</commit_message>
<xml_diff>
--- a/where to start coding - notes from the last session.xlsx
+++ b/where to start coding - notes from the last session.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06FAA6F-033B-4501-98A2-53386AAA4F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D170AB-3532-4DFB-9B48-11FB73CB04CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Date of Coding</t>
   </si>
@@ -75,6 +75,18 @@
   </si>
   <si>
     <t xml:space="preserve">The 2023 veg data was exported, raw without manipulation, into folder "summary output" as df = "veg2023_raw(19july2025)" from file="test_2023_regen_plot_input.Rmd".  Read that data into "slash_veg_complete.Rmd" at line 416 and calculate the stems per acre and "clumps_per acre" and "ramets_clump". Check the plot radius coefficients on line 407 The code for the clump and ramet calculations are likely available on line ~469 for df=veg2024 and have been confirmed.  </t>
+  </si>
+  <si>
+    <t>start with df = regen2024_updated on line=1537</t>
+  </si>
+  <si>
+    <t>july 22 2024</t>
+  </si>
+  <si>
+    <t>revised regen2023 and regen2024</t>
+  </si>
+  <si>
+    <t>untangle seedA which are commercial species that are input into df=seedlings2019_2024 for use in df=sitedata. See line 1171.  go back through all the regen data and validate the labels used and conversions to common notation as A, B, C, D, and sapl.  seedA is for commercial seedlings and makes sense for a metric in the site data, but the 4-12" data is needed for the veg01data and seedA is not needed.</t>
   </si>
 </sst>
 </file>
@@ -476,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10441F4B-E333-43AC-9DFC-8056F26DEB96}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" customWidth="1"/>
@@ -536,6 +548,22 @@
         <v>12</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="103.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
resolved and confirmed that seedA was the per acre value of commercial species, which excludes black birch. Also that all of the seedling height class labels were correctly applied.
</commit_message>
<xml_diff>
--- a/where to start coding - notes from the last session.xlsx
+++ b/where to start coding - notes from the last session.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D170AB-3532-4DFB-9B48-11FB73CB04CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C8BA14-B7CB-414E-B2F0-9249308AB7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Date of Coding</t>
   </si>
@@ -80,13 +80,25 @@
     <t>start with df = regen2024_updated on line=1537</t>
   </si>
   <si>
-    <t>july 22 2024</t>
-  </si>
-  <si>
     <t>revised regen2023 and regen2024</t>
   </si>
   <si>
     <t>untangle seedA which are commercial species that are input into df=seedlings2019_2024 for use in df=sitedata. See line 1171.  go back through all the regen data and validate the labels used and conversions to common notation as A, B, C, D, and sapl.  seedA is for commercial seedlings and makes sense for a metric in the site data, but the 4-12" data is needed for the veg01data and seedA is not needed.</t>
+  </si>
+  <si>
+    <t>july 23 2025</t>
+  </si>
+  <si>
+    <t>july 22 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1) determine if there are seedA data for cafri in 2022.  those value are NA for veg01 which builds from veg_complete_2019_2022. (cafri veg data exist in 2022, but need to check the df=site_data and if that made it into the df~=pre2023seedling. (2) determine why in df=veg01, I use on line 1490 a full_join of seedlings2019_2024 to a df complete through 2022? (3) determine if I need to add "type" labels line 1512, those might be present (4) on line 1744 for df=yay, assess if I should use "bind_row" or left_join to bring in the 2023 and 2024 regen_updated df. </t>
+  </si>
+  <si>
+    <t>resolved and confirmed that seedA was the per acre value of commercial species, which excludes black birch. Also that all of the seedling height class labels were correctly applied.</t>
+  </si>
+  <si>
+    <t>july 24 2025</t>
   </si>
 </sst>
 </file>
@@ -133,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -149,9 +161,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -488,22 +497,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10441F4B-E333-43AC-9DFC-8056F26DEB96}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="62.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="78" style="3" customWidth="1"/>
+    <col min="3" max="3" width="78" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
     </row>
@@ -514,6 +523,7 @@
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -550,18 +560,32 @@
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="103.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="103.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C8" s="2" t="s">
-        <v>16</v>
+    </row>
+    <row r="9" spans="1:3" ht="112.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mostly updated the creation of df=yay
</commit_message>
<xml_diff>
--- a/where to start coding - notes from the last session.xlsx
+++ b/where to start coding - notes from the last session.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C8BA14-B7CB-414E-B2F0-9249308AB7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F117A79D-9612-4BCB-A3CA-895D093A5217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Date of Coding</t>
   </si>
@@ -99,6 +100,15 @@
   </si>
   <si>
     <t>july 24 2025</t>
+  </si>
+  <si>
+    <t>Item #4 above from 24 july is done. The remainder of items 1 - 3 need attention.</t>
+  </si>
+  <si>
+    <t>july 25 2025</t>
+  </si>
+  <si>
+    <t>creation of df=yay</t>
   </si>
 </sst>
 </file>
@@ -497,7 +507,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10441F4B-E333-43AC-9DFC-8056F26DEB96}">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" style="1" customWidth="1"/>
@@ -588,6 +598,17 @@
         <v>18</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
worked on making sure seedA was present throughout especiall 2019 thru 2022
</commit_message>
<xml_diff>
--- a/where to start coding - notes from the last session.xlsx
+++ b/where to start coding - notes from the last session.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F117A79D-9612-4BCB-A3CA-895D093A5217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5982C1E8-8610-4DA7-8FCD-EBB123574448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Date of Coding</t>
   </si>
@@ -109,6 +108,18 @@
   </si>
   <si>
     <t>creation of df=yay</t>
+  </si>
+  <si>
+    <t>sort</t>
+  </si>
+  <si>
+    <t>july 28 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">completed #1 from july 25 such that seedA is present in all years.  Resolved #2 with left_join. </t>
+  </si>
+  <si>
+    <t>check if "type" labels are needed in df = yay.  Check data to make sure the values seem reasonable…not sure how to do this.</t>
   </si>
 </sst>
 </file>
@@ -155,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -173,6 +184,25 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,109 +537,157 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10441F4B-E333-43AC-9DFC-8056F26DEB96}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="62.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="78" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="12"/>
+    <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="62.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="78" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:4" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" s="3" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+    <row r="2" spans="1:4" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+    </row>
+    <row r="3" spans="1:4" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="11"/>
+      <c r="B3" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="3" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="12">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="117.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="12">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="148.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="125.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12">
+        <v>4</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="103.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="12">
+        <v>3</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="112.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12">
+        <v>2</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13">
+        <v>1</v>
+      </c>
+      <c r="B11" s="1">
         <v>45852</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:3" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="148.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="125.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="103.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="112.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>21</v>
-      </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D11">
+    <sortCondition descending="1" ref="A4:A11"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
making the data complete for all seasons. replace df=yay with df=yay2
</commit_message>
<xml_diff>
--- a/where to start coding - notes from the last session.xlsx
+++ b/where to start coding - notes from the last session.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5982C1E8-8610-4DA7-8FCD-EBB123574448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD9FE951-3234-4E8A-9A13-C4B209761187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="suggested checks on df=yay2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="53">
   <si>
     <t>Date of Coding</t>
   </si>
@@ -120,6 +121,101 @@
   </si>
   <si>
     <t>check if "type" labels are needed in df = yay.  Check data to make sure the values seem reasonable…not sure how to do this.</t>
+  </si>
+  <si>
+    <t>1. Species Completeness Consistency</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>CopyEdit</t>
+  </si>
+  <si>
+    <t>yay2 %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  group_by(season, wall) %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  summarize(n_points = n_distinct(point), n_species = n_distinct(spp)) %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  arrange(desc(n_species)) # Or look at min/max</t>
+  </si>
+  <si>
+    <t>2. Point × Species Grid Completeness</t>
+  </si>
+  <si>
+    <t>You could cross-tabulate the expected vs. actual grid size:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  summarize(</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    expected = n_distinct(point) * n_distinct(spp),</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    actual = n()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ) %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  filter(actual != expected)</t>
+  </si>
+  <si>
+    <t>3. Missing Value Sanity Check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  summarize(across(everything(), ~ sum(is.na(.)))) %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  pivot_longer(everything()) %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  filter(value &gt; 0)</t>
+  </si>
+  <si>
+    <t>4. Species Distribution by Season</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Confirm that each </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>spp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> appears as expected:</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">  count(season, spp) %&gt;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  pivot_wider(names_from = spp, values_from = n, values_fill = 0)</t>
+  </si>
+  <si>
+    <t>july 29 2025</t>
+  </si>
+  <si>
+    <t>made all seasons complete</t>
+  </si>
+  <si>
+    <t>1. figure out the spp = na for df=errro_check. All exist in season 2024.  2. search for points that include "emplty" and other species. Remove the record for "empty". 3. run the check provided by chatgpt on the next worksheet.</t>
   </si>
 </sst>
 </file>
@@ -129,7 +225,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,6 +240,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -166,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -184,24 +285,23 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -538,16 +638,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10441F4B-E333-43AC-9DFC-8056F26DEB96}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="12"/>
+    <col min="1" max="1" width="9.140625" style="8"/>
     <col min="2" max="2" width="22.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="62.7109375" style="2" customWidth="1"/>
     <col min="4" max="4" width="78" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="6" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:4" s="6" customFormat="1" ht="15" customHeight="1">
+      <c r="A1" s="7" t="s">
         <v>24</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -560,26 +660,30 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-    </row>
-    <row r="3" spans="1:4" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11"/>
-      <c r="B3" s="8" t="s">
+    <row r="2" spans="1:4" ht="78" customHeight="1">
+      <c r="B2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="59.25" customHeight="1">
+      <c r="B3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="3" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12">
+    <row r="4" spans="1:4" s="3" customFormat="1" ht="52.5" customHeight="1">
+      <c r="A4" s="8">
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -592,8 +696,8 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="117.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12">
+    <row r="5" spans="1:4" ht="117.75" customHeight="1">
+      <c r="A5" s="8">
         <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -606,8 +710,8 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="148.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12">
+    <row r="6" spans="1:4" ht="148.5" customHeight="1">
+      <c r="A6" s="8">
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -617,8 +721,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="125.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12">
+    <row r="7" spans="1:4" ht="125.25" customHeight="1">
+      <c r="A7" s="8">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -631,8 +735,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12">
+    <row r="8" spans="1:4" ht="15" customHeight="1">
+      <c r="A8" s="8">
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -645,8 +749,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="103.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12">
+    <row r="9" spans="1:4" ht="103.5" customHeight="1">
+      <c r="A9" s="8">
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -659,8 +763,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="112.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12">
+    <row r="10" spans="1:4" ht="112.5" customHeight="1">
+      <c r="A10" s="8">
         <v>2</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -673,8 +777,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="13">
+    <row r="11" spans="1:4" ht="15" customHeight="1">
+      <c r="A11" s="9">
         <v>1</v>
       </c>
       <c r="B11" s="1">
@@ -691,4 +795,198 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA27206A-E7F3-4443-8D50-6F1C81479A5D}">
+  <dimension ref="A1:A39"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="82" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="3"/>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="10"/>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="3"/>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" s="12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" s="12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" s="12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" s="12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" s="12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" s="10"/>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" s="11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" s="3"/>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" s="12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" s="12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" s="12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" s="12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" s="10"/>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" s="3"/>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" s="12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" s="12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" s="12" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
tested the final data. looks good except for clumps/acre and stems/ramet. The original data was saved_as *_OLD.Rmd
</commit_message>
<xml_diff>
--- a/where to start coding - notes from the last session.xlsx
+++ b/where to start coding - notes from the last session.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD9FE951-3234-4E8A-9A13-C4B209761187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9071686C-DDD7-4BE5-AD9B-60416441F69C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
started working through the df for analysis of data.
</commit_message>
<xml_diff>
--- a/where to start coding - notes from the last session.xlsx
+++ b/where to start coding - notes from the last session.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9071686C-DDD7-4BE5-AD9B-60416441F69C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB402EB7-28AE-46C2-AB9E-D7C26B551322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="58">
   <si>
     <t>Date of Coding</t>
   </si>
@@ -216,6 +216,21 @@
   </si>
   <si>
     <t>1. figure out the spp = na for df=errro_check. All exist in season 2024.  2. search for points that include "emplty" and other species. Remove the record for "empty". 3. run the check provided by chatgpt on the next worksheet.</t>
+  </si>
+  <si>
+    <t>july 31 2025</t>
+  </si>
+  <si>
+    <t>start on df-d1.1 and make sure the summarize statement is correct.</t>
+  </si>
+  <si>
+    <t>minor mop up from the complete data set</t>
+  </si>
+  <si>
+    <t>working through the calculations of df=slash_wall_analyses_2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1) think about what you want from the df=type_summary and df=wall_type_occupancy. These produce the percentage of points within a harvest x type where a type is present, by the three categories (any, &gt;1 ft, &gt;5 ft). The calculations seem valid. Include "brush" in the "by" groupings. complete test calculations from df=d1_stub (2) define denominator and type_count in df=type_summary (3) start reviewing df=species_by_wall  </t>
   </si>
 </sst>
 </file>
@@ -267,7 +282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -303,6 +318,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -637,7 +662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10441F4B-E333-43AC-9DFC-8056F26DEB96}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="8"/>
@@ -660,137 +685,161 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="78" customHeight="1">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="1:4" s="16" customFormat="1" ht="117" customHeight="1">
+      <c r="A2" s="13"/>
+      <c r="B2" s="14">
+        <v>45870</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="16" customFormat="1" ht="120.75" customHeight="1">
+      <c r="A3" s="13"/>
+      <c r="B3" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="78" customHeight="1">
+      <c r="B4" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="59.25" customHeight="1">
-      <c r="B3" s="1" t="s">
+    <row r="5" spans="1:4" ht="59.25" customHeight="1">
+      <c r="B5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="3" customFormat="1" ht="52.5" customHeight="1">
-      <c r="A4" s="8">
+    <row r="6" spans="1:4" s="3" customFormat="1" ht="52.5" customHeight="1">
+      <c r="A6" s="8">
         <v>8</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="117.75" customHeight="1">
-      <c r="A5" s="8">
+    <row r="7" spans="1:4" ht="117.75" customHeight="1">
+      <c r="A7" s="8">
         <v>7</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="148.5" customHeight="1">
-      <c r="A6" s="8">
+    <row r="8" spans="1:4" ht="148.5" customHeight="1">
+      <c r="A8" s="8">
         <v>6</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="125.25" customHeight="1">
-      <c r="A7" s="8">
+    <row r="9" spans="1:4" ht="125.25" customHeight="1">
+      <c r="A9" s="8">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15" customHeight="1">
-      <c r="A8" s="8">
+    <row r="10" spans="1:4" ht="15" customHeight="1">
+      <c r="A10" s="8">
         <v>4</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="103.5" customHeight="1">
-      <c r="A9" s="8">
+    <row r="11" spans="1:4" ht="103.5" customHeight="1">
+      <c r="A11" s="8">
         <v>3</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="112.5" customHeight="1">
-      <c r="A10" s="8">
+    <row r="12" spans="1:4" ht="112.5" customHeight="1">
+      <c r="A12" s="8">
         <v>2</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15" customHeight="1">
-      <c r="A11" s="9">
+    <row r="13" spans="1:4" ht="15" customHeight="1">
+      <c r="A13" s="9">
         <v>1</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B13" s="1">
         <v>45852</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D11">
-    <sortCondition descending="1" ref="A4:A11"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:D13">
+    <sortCondition descending="1" ref="A6:A13"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
mostly worked on type_summary and richness calculations
</commit_message>
<xml_diff>
--- a/where to start coding - notes from the last session.xlsx
+++ b/where to start coding - notes from the last session.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjs23\Documents\R\slash-wall-vegetation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB402EB7-28AE-46C2-AB9E-D7C26B551322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECEFD680-A5E2-4D50-A7CE-B79CE0F582B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C3CAF665-40FD-431B-82A7-2BF54862B878}"/>
   </bookViews>
@@ -230,7 +230,7 @@
     <t>working through the calculations of df=slash_wall_analyses_2025</t>
   </si>
   <si>
-    <t xml:space="preserve">(1) think about what you want from the df=type_summary and df=wall_type_occupancy. These produce the percentage of points within a harvest x type where a type is present, by the three categories (any, &gt;1 ft, &gt;5 ft). The calculations seem valid. Include "brush" in the "by" groupings. complete test calculations from df=d1_stub (2) define denominator and type_count in df=type_summary (3) start reviewing df=species_by_wall  </t>
+    <t xml:space="preserve">(0) write up a little summary for each df to explain why the calculations are made. (1) think about what you want from the df=type_summary and df=wall_type_occupancy. These produce the percentage of points within a harvest x type where a type is present, by the three categories (any, &gt;1 ft, &gt;5 ft). The calculations seem valid. Include "brush" in the "by" groupings. complete test calculations from df=d1_stub (2) define denominator and type_count in df=type_summary (3) start reviewing df=species_by_wall  </t>
   </si>
 </sst>
 </file>

</xml_diff>